<commit_message>
updated constraints for product inclusion in catalog to keep things in OVAP
</commit_message>
<xml_diff>
--- a/output/SKUs Removed From Catalog - 260511.xlsx
+++ b/output/SKUs Removed From Catalog - 260511.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -435,13 +435,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>OM3S</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>